<commit_message>
Updated ADLD_dup_1 coordinates and deleted test cells
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Publication" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="184">
   <si>
     <t xml:space="preserve">Item name</t>
   </si>
@@ -156,9 +156,6 @@
     <t xml:space="preserve">ADLD_dup_13</t>
   </si>
   <si>
-    <t xml:space="preserve">test</t>
-  </si>
-  <si>
     <t xml:space="preserve">ADLD_dup_14</t>
   </si>
   <si>
@@ -541,9 +538,6 @@
   </si>
   <si>
     <t xml:space="preserve">Microhomolgy of GA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEST</t>
   </si>
   <si>
     <t xml:space="preserve">n/a</t>
@@ -1146,16 +1140,14 @@
       <c r="A14" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>44</v>
-      </c>
+      <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="3"/>
     </row>
     <row r="15" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1164,7 +1156,7 @@
     </row>
     <row r="16" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1173,22 +1165,22 @@
     </row>
     <row r="17" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="E17" s="3"/>
     </row>
     <row r="18" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="5"/>
@@ -1197,24 +1189,24 @@
     </row>
     <row r="19" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="E19" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="5"/>
@@ -1223,39 +1215,39 @@
     </row>
     <row r="21" s="4" customFormat="true" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="22" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="E22" s="3"/>
     </row>
     <row r="23" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>24</v>
@@ -1264,63 +1256,63 @@
         <v>25</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E23" s="3"/>
     </row>
     <row r="24" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="3"/>
     </row>
     <row r="25" s="4" customFormat="true" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>73</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>74</v>
       </c>
       <c r="E25" s="3"/>
     </row>
     <row r="26" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="3"/>
     </row>
     <row r="27" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="C27" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>31</v>
@@ -1328,7 +1320,7 @@
     </row>
     <row r="28" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1337,16 +1329,16 @@
     </row>
     <row r="29" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>84</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>31</v>
@@ -1354,7 +1346,7 @@
     </row>
     <row r="30" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>24</v>
@@ -1363,65 +1355,65 @@
         <v>25</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E30" s="3"/>
     </row>
     <row r="31" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="C31" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="D31" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="32" s="4" customFormat="true" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="C32" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="33" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>25</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E33" s="3"/>
     </row>
     <row r="34" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" s="5" t="s">
         <v>99</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>100</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5"/>
@@ -1429,20 +1421,20 @@
     </row>
     <row r="35" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="D35" s="5"/>
       <c r="E35" s="3"/>
     </row>
     <row r="36" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="5"/>
@@ -1451,25 +1443,25 @@
     </row>
     <row r="37" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>105</v>
       </c>
       <c r="E37" s="3"/>
     </row>
     <row r="38" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
@@ -1477,42 +1469,42 @@
     </row>
     <row r="39" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E39" s="3"/>
     </row>
     <row r="40" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B40" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="C40" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="E40" s="3"/>
     </row>
     <row r="41" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D41" s="5" t="s">
         <v>114</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>115</v>
       </c>
       <c r="E41" s="3"/>
     </row>
@@ -1827,16 +1819,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="7" t="s">
         <v>118</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="2" s="4" customFormat="true" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1844,14 +1836,14 @@
         <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>16</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" s="4" customFormat="true" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1859,7 +1851,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>31</v>
@@ -1868,7 +1860,7 @@
         <v>45</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" s="4" customFormat="true" ht="77.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1876,7 +1868,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>3</v>
@@ -1885,7 +1877,7 @@
         <v>43</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1893,14 +1885,14 @@
         <v>19</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>3</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1908,7 +1900,7 @@
         <v>23</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
@@ -1919,16 +1911,16 @@
         <v>27</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="D7" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="E7" s="7" t="s">
         <v>130</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="8" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1936,7 +1928,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
@@ -1947,16 +1939,16 @@
         <v>34</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>4</v>
       </c>
       <c r="D9" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>133</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="10" s="4" customFormat="true" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1964,16 +1956,16 @@
         <v>37</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>4</v>
       </c>
       <c r="D10" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>136</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="11" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1981,7 +1973,7 @@
         <v>39</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
@@ -2016,7 +2008,7 @@
     </row>
     <row r="15" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="11"/>
@@ -2025,10 +2017,10 @@
     </row>
     <row r="16" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
@@ -2036,20 +2028,20 @@
     </row>
     <row r="17" s="4" customFormat="true" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="11"/>
       <c r="D17" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="E17" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="18" s="4" customFormat="true" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="11"/>
@@ -2057,12 +2049,12 @@
         <v>52</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="11"/>
@@ -2071,10 +2063,10 @@
     </row>
     <row r="20" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
@@ -2082,10 +2074,10 @@
     </row>
     <row r="21" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
@@ -2093,7 +2085,7 @@
     </row>
     <row r="22" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="11"/>
@@ -2102,7 +2094,7 @@
     </row>
     <row r="23" s="4" customFormat="true" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="11"/>
@@ -2110,23 +2102,23 @@
         <v>34</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" s="4" customFormat="true" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
       <c r="E24" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="11"/>
@@ -2135,10 +2127,10 @@
     </row>
     <row r="26" s="4" customFormat="true" ht="77.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>2</v>
@@ -2147,15 +2139,15 @@
         <v>48</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" s="4" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
@@ -2163,10 +2155,10 @@
     </row>
     <row r="28" s="4" customFormat="true" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C28" s="10" t="n">
         <v>12</v>
@@ -2175,29 +2167,29 @@
         <v>45</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" s="4" customFormat="true" ht="77.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C29" s="10" t="n">
         <v>8</v>
       </c>
       <c r="D29" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="E29" s="7" t="s">
         <v>150</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="30" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="11"/>
@@ -2206,7 +2198,7 @@
     </row>
     <row r="31" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="11"/>
@@ -2215,7 +2207,7 @@
     </row>
     <row r="32" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="11"/>
@@ -2224,18 +2216,18 @@
     </row>
     <row r="33" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="11"/>
       <c r="D33" s="11"/>
       <c r="E33" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="34" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="11"/>
@@ -2244,7 +2236,7 @@
     </row>
     <row r="35" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="11"/>
@@ -2253,7 +2245,7 @@
     </row>
     <row r="36" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="11"/>
@@ -2587,22 +2579,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="E1" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="3" t="s">
         <v>157</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="2" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2610,22 +2602,22 @@
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C2" s="15" t="n">
-        <v>127204606</v>
+        <v>126687731</v>
       </c>
       <c r="D2" s="15" t="n">
-        <v>127486761</v>
+        <v>126965660</v>
       </c>
       <c r="E2" s="15" t="n">
         <v>277929</v>
       </c>
       <c r="F2" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>160</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="3" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2633,7 +2625,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C3" s="15" t="n">
         <v>126736375</v>
@@ -2645,10 +2637,10 @@
         <v>203432</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2656,7 +2648,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4" s="14" t="n">
         <v>126742343</v>
@@ -2668,10 +2660,10 @@
         <v>189731</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2679,7 +2671,7 @@
         <v>19</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>126763901</v>
@@ -2691,10 +2683,10 @@
         <v>150283</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2702,7 +2694,7 @@
         <v>23</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>126683194</v>
@@ -2714,10 +2706,10 @@
         <v>238941</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2725,7 +2717,7 @@
         <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C7" s="15" t="n">
         <v>126761184</v>
@@ -2734,13 +2726,13 @@
         <v>126930640</v>
       </c>
       <c r="E7" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="F7" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="G7" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="8" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2748,7 +2740,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>126667591</v>
@@ -2760,10 +2752,10 @@
         <v>340785</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2771,7 +2763,7 @@
         <v>34</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>126705616</v>
@@ -2783,10 +2775,10 @@
         <v>203842</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2794,7 +2786,7 @@
         <v>37</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C10" s="14" t="n">
         <v>126686881</v>
@@ -2806,10 +2798,10 @@
         <v>228672</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2817,7 +2809,7 @@
         <v>39</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C11" s="14" t="n">
         <v>126766751</v>
@@ -2829,10 +2821,10 @@
         <v>229243</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2840,7 +2832,7 @@
         <v>41</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C12" s="15" t="n">
         <v>126687731</v>
@@ -2848,9 +2840,7 @@
       <c r="D12" s="15" t="n">
         <v>126965660</v>
       </c>
-      <c r="E12" s="15" t="s">
-        <v>173</v>
-      </c>
+      <c r="E12" s="15"/>
       <c r="F12" s="11"/>
       <c r="G12" s="5"/>
     </row>
@@ -2859,7 +2849,7 @@
         <v>42</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C13" s="15" t="n">
         <v>126775269</v>
@@ -2876,7 +2866,7 @@
         <v>43</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C14" s="15" t="n">
         <v>126716573</v>
@@ -2890,10 +2880,10 @@
     </row>
     <row r="15" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C15" s="15" t="n">
         <v>126743135</v>
@@ -2907,10 +2897,10 @@
     </row>
     <row r="16" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C16" s="15" t="n">
         <v>125918128</v>
@@ -2924,10 +2914,10 @@
     </row>
     <row r="17" s="4" customFormat="true" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C17" s="14" t="n">
         <v>126016772</v>
@@ -2939,18 +2929,18 @@
         <v>672515</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C18" s="14" t="n">
         <v>126050112</v>
@@ -2964,10 +2954,10 @@
     </row>
     <row r="19" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C19" s="14" t="n">
         <v>126156719</v>
@@ -2979,18 +2969,18 @@
         <v>609000</v>
       </c>
       <c r="F19" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>174</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="20" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C20" s="14" t="n">
         <v>126156745</v>
@@ -3004,10 +2994,10 @@
     </row>
     <row r="21" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C21" s="14" t="n">
         <v>126363827</v>
@@ -3019,18 +3009,18 @@
         <v>474998</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="22" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C22" s="15" t="n">
         <v>126512007</v>
@@ -3044,10 +3034,10 @@
     </row>
     <row r="23" s="4" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C23" s="14" t="n">
         <v>126522203</v>
@@ -3059,18 +3049,18 @@
         <v>250000</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" s="4" customFormat="true" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C24" s="14" t="n">
         <v>126695490</v>
@@ -3082,18 +3072,18 @@
         <v>340785</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C25" s="14" t="n">
         <v>126698430</v>
@@ -3107,10 +3097,10 @@
     </row>
     <row r="26" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C26" s="14" t="n">
         <v>126705102</v>
@@ -3122,18 +3112,18 @@
         <v>324675</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C27" s="14" t="n">
         <v>126713540</v>
@@ -3145,18 +3135,18 @@
         <v>234020</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C28" s="14" t="n">
         <v>126718880</v>
@@ -3168,18 +3158,18 @@
         <v>148085</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="29" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C29" s="14" t="n">
         <v>126732318</v>
@@ -3191,18 +3181,18 @@
         <v>153769</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C30" s="14" t="n">
         <v>126736453</v>
@@ -3214,18 +3204,18 @@
         <v>127608</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C31" s="14" t="n">
         <v>126739243</v>
@@ -3239,10 +3229,10 @@
     </row>
     <row r="32" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C32" s="14" t="n">
         <v>126753827</v>
@@ -3256,10 +3246,10 @@
     </row>
     <row r="33" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C33" s="14" t="n">
         <v>126763765</v>
@@ -3275,10 +3265,10 @@
     </row>
     <row r="34" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C34" s="14" t="n">
         <v>126766199</v>
@@ -3292,10 +3282,10 @@
     </row>
     <row r="35" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C35" s="14" t="n">
         <v>126762001</v>
@@ -3309,10 +3299,10 @@
     </row>
     <row r="36" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C36" s="14" t="n">
         <v>126805047</v>

</xml_diff>

<commit_message>
Updated the Evidence tab to only have one column
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C72D020-47C9-4E62-9997-0FF7B23BA7BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2388684B-CA99-4C5B-AD67-D7724DF1017F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Molecular" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="262">
   <si>
     <t>Item name</t>
   </si>
@@ -701,19 +701,130 @@
     <t>NonADLD_dup_6</t>
   </si>
   <si>
-    <t>Publications</t>
-  </si>
-  <si>
-    <t>Literature case labels</t>
-  </si>
-  <si>
-    <t>Multigenerational families</t>
-  </si>
-  <si>
-    <t>Estimated unique affected individuals</t>
-  </si>
-  <si>
-    <t>Deduplication status</t>
+    <t>Summarry</t>
+  </si>
+  <si>
+    <t>Testing 1</t>
+  </si>
+  <si>
+    <t>Testing 2</t>
+  </si>
+  <si>
+    <t>Testing 3</t>
+  </si>
+  <si>
+    <t>Testing 4</t>
+  </si>
+  <si>
+    <t>Testing 5</t>
+  </si>
+  <si>
+    <t>Testing 6</t>
+  </si>
+  <si>
+    <t>Testing 7</t>
+  </si>
+  <si>
+    <t>Testing 8</t>
+  </si>
+  <si>
+    <t>Testing 9</t>
+  </si>
+  <si>
+    <t>Testing 10</t>
+  </si>
+  <si>
+    <t>Testing 11</t>
+  </si>
+  <si>
+    <t>Testing 12</t>
+  </si>
+  <si>
+    <t>Testing 13</t>
+  </si>
+  <si>
+    <t>Testing 14</t>
+  </si>
+  <si>
+    <t>Testing 15</t>
+  </si>
+  <si>
+    <t>Testing 16</t>
+  </si>
+  <si>
+    <t>Testing 17</t>
+  </si>
+  <si>
+    <t>Testing 18</t>
+  </si>
+  <si>
+    <t>Testing 19</t>
+  </si>
+  <si>
+    <t>Testing 20</t>
+  </si>
+  <si>
+    <t>Testing 21</t>
+  </si>
+  <si>
+    <t>Testing 22</t>
+  </si>
+  <si>
+    <t>Testing 23</t>
+  </si>
+  <si>
+    <t>Testing 24</t>
+  </si>
+  <si>
+    <t>Testing 25</t>
+  </si>
+  <si>
+    <t>Testing 26</t>
+  </si>
+  <si>
+    <t>Testing 27</t>
+  </si>
+  <si>
+    <t>Testing 28</t>
+  </si>
+  <si>
+    <t>Testing 29</t>
+  </si>
+  <si>
+    <t>Testing 30</t>
+  </si>
+  <si>
+    <t>Testing 31</t>
+  </si>
+  <si>
+    <t>Testing 32</t>
+  </si>
+  <si>
+    <t>Testing 33</t>
+  </si>
+  <si>
+    <t>Testing 34</t>
+  </si>
+  <si>
+    <t>Testing 35</t>
+  </si>
+  <si>
+    <t>Testing 36</t>
+  </si>
+  <si>
+    <t>Testing 37</t>
+  </si>
+  <si>
+    <t>Testing 38</t>
+  </si>
+  <si>
+    <t>Testing 39</t>
+  </si>
+  <si>
+    <t>Testing 40</t>
+  </si>
+  <si>
+    <t>Testing 41</t>
   </si>
 </sst>
 </file>
@@ -724,7 +835,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -751,6 +862,12 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1982,904 +2099,351 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93210A17-976E-449D-A8F5-248F94CB6DA5}">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="104.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="95.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="2">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2">
-        <v>126965629</v>
-      </c>
-      <c r="D2" s="2">
-        <v>126966115</v>
-      </c>
-      <c r="E2" s="2">
-        <v>277929</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2">
-        <v>126736375</v>
-      </c>
-      <c r="D3" s="2">
-        <v>126939807</v>
-      </c>
-      <c r="E3" s="2">
-        <v>203432</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="2">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2">
-        <v>126742343</v>
-      </c>
-      <c r="D4" s="2">
-        <v>126932074</v>
-      </c>
-      <c r="E4" s="2">
-        <v>189731</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="2">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2">
-        <v>126763901</v>
-      </c>
-      <c r="D5" s="2">
-        <v>126914184</v>
-      </c>
-      <c r="E5" s="2">
-        <v>150283</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="2">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2">
-        <v>126683194</v>
-      </c>
-      <c r="D6" s="2">
-        <v>126922135</v>
-      </c>
-      <c r="E6" s="2">
-        <v>238941</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="2">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2">
-        <v>126761184</v>
-      </c>
-      <c r="D7" s="2">
-        <v>126930640</v>
-      </c>
-      <c r="E7" s="2">
-        <v>169456</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="2">
-        <v>5</v>
-      </c>
-      <c r="C8" s="2">
-        <v>126667591</v>
-      </c>
-      <c r="D8" s="2">
-        <v>127008376</v>
-      </c>
-      <c r="E8" s="2">
-        <v>340785</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="2">
-        <v>5</v>
-      </c>
-      <c r="C9" s="2">
-        <v>126705616</v>
-      </c>
-      <c r="D9" s="2">
-        <v>126909458</v>
-      </c>
-      <c r="E9" s="2">
-        <v>203842</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="2">
-        <v>5</v>
-      </c>
-      <c r="C10" s="2">
-        <v>126686881</v>
-      </c>
-      <c r="D10" s="2">
-        <v>126915553</v>
-      </c>
-      <c r="E10" s="2">
-        <v>228672</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="2">
-        <v>5</v>
-      </c>
-      <c r="C11" s="2">
-        <v>126766751</v>
-      </c>
-      <c r="D11" s="2">
-        <v>126995994</v>
-      </c>
-      <c r="E11" s="2">
-        <v>229243</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B12" s="2">
-        <v>5</v>
-      </c>
-      <c r="C12" s="2">
-        <v>126687731</v>
-      </c>
-      <c r="D12" s="2">
-        <v>126965660</v>
-      </c>
-      <c r="E12" s="2">
-        <v>277929</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B13" s="2">
-        <v>5</v>
-      </c>
-      <c r="C13" s="2">
-        <v>126775269</v>
-      </c>
-      <c r="D13" s="2">
-        <v>126893623</v>
-      </c>
-      <c r="E13" s="2">
-        <v>118354</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="2">
-        <v>5</v>
-      </c>
-      <c r="C14" s="2">
-        <v>126716573</v>
-      </c>
-      <c r="D14" s="2">
-        <v>126926882</v>
-      </c>
-      <c r="E14" s="2">
-        <v>210309</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B15" s="2">
-        <v>5</v>
-      </c>
-      <c r="C15" s="2">
-        <v>126743135</v>
-      </c>
-      <c r="D15" s="2">
-        <v>126865131</v>
-      </c>
-      <c r="E15" s="2">
-        <v>121996</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B16" s="2">
-        <v>5</v>
-      </c>
-      <c r="C16" s="2">
-        <v>125918128</v>
-      </c>
-      <c r="D16" s="2">
-        <v>126949480</v>
-      </c>
-      <c r="E16" s="2">
-        <v>1031351</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="2">
-        <v>5</v>
-      </c>
-      <c r="C17" s="2">
-        <v>126016772</v>
-      </c>
-      <c r="D17" s="2">
-        <v>126689287</v>
-      </c>
-      <c r="E17" s="2">
-        <v>672515</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B18" s="2">
-        <v>5</v>
-      </c>
-      <c r="C18" s="2">
-        <v>122477418</v>
-      </c>
-      <c r="D18" s="2">
-        <v>126843396</v>
-      </c>
-      <c r="E18" s="2">
-        <v>4365976</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B19" s="2">
-        <v>5</v>
-      </c>
-      <c r="C19" s="2">
-        <v>122477254</v>
-      </c>
-      <c r="D19" s="2">
-        <v>126843256</v>
-      </c>
-      <c r="E19" s="2">
-        <v>4366000</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B20" s="2">
-        <v>5</v>
-      </c>
-      <c r="C20" s="2">
-        <v>122476520</v>
-      </c>
-      <c r="D20" s="2">
-        <v>126842588</v>
-      </c>
-      <c r="E20" s="2">
-        <v>4366065</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="2">
-        <v>5</v>
-      </c>
-      <c r="C21" s="2">
-        <v>126050112</v>
-      </c>
-      <c r="D21" s="2">
-        <v>126707361</v>
-      </c>
-      <c r="E21" s="2">
-        <v>660000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="2">
-        <v>5</v>
-      </c>
-      <c r="C22" s="2">
-        <v>126156719</v>
-      </c>
-      <c r="D22" s="2">
-        <v>126765604</v>
-      </c>
-      <c r="E22" s="2">
-        <v>608833</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B23" s="2">
-        <v>5</v>
-      </c>
-      <c r="C23" s="2">
-        <v>126363827</v>
-      </c>
-      <c r="D23" s="2">
-        <v>126838825</v>
-      </c>
-      <c r="E23" s="2">
-        <v>474998</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B24" s="2">
-        <v>5</v>
-      </c>
-      <c r="C24" s="2">
-        <v>126512007</v>
-      </c>
-      <c r="D24" s="2">
-        <v>126978629</v>
-      </c>
-      <c r="E24" s="2">
-        <v>466623</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B25" s="2">
-        <v>5</v>
-      </c>
-      <c r="C25" s="2">
-        <v>126522203</v>
-      </c>
-      <c r="D25" s="2">
-        <v>126772687</v>
-      </c>
-      <c r="E25" s="2">
-        <v>250000</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B26" s="2">
-        <v>5</v>
-      </c>
-      <c r="C26" s="2">
-        <v>126637847</v>
-      </c>
-      <c r="D26" s="2">
-        <v>126913193</v>
-      </c>
-      <c r="E26" s="2">
-        <v>275347</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B27" s="2">
-        <v>5</v>
-      </c>
-      <c r="C27" s="2">
-        <v>126695490</v>
-      </c>
-      <c r="D27" s="2">
-        <v>127036275</v>
-      </c>
-      <c r="E27" s="2">
-        <v>340785</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B28" s="2">
-        <v>5</v>
-      </c>
-      <c r="C28" s="2">
-        <v>126698430</v>
-      </c>
-      <c r="D28" s="2">
-        <v>126889630</v>
-      </c>
-      <c r="E28" s="2">
-        <v>191200</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B29" s="2">
-        <v>5</v>
-      </c>
-      <c r="C29" s="2">
-        <v>126705102</v>
-      </c>
-      <c r="D29" s="2">
-        <v>127029777</v>
-      </c>
-      <c r="E29" s="2">
-        <v>324675</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B30" s="2">
-        <v>5</v>
-      </c>
-      <c r="C30" s="2">
-        <v>126713540</v>
-      </c>
-      <c r="D30" s="2">
-        <v>126947560</v>
-      </c>
-      <c r="E30" s="2">
-        <v>234020</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B31" s="2">
-        <v>5</v>
-      </c>
-      <c r="C31" s="2">
-        <v>126718880</v>
-      </c>
-      <c r="D31" s="2">
-        <v>126866965</v>
-      </c>
-      <c r="E31" s="2">
-        <v>148085</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B32" s="2">
-        <v>5</v>
-      </c>
-      <c r="C32" s="2">
-        <v>126732318</v>
-      </c>
-      <c r="D32" s="2">
-        <v>126886087</v>
-      </c>
-      <c r="E32" s="2">
-        <v>153769</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B33" s="2">
-        <v>5</v>
-      </c>
-      <c r="C33" s="2">
-        <v>126736453</v>
-      </c>
-      <c r="D33" s="2">
-        <v>126864061</v>
-      </c>
-      <c r="E33" s="2">
-        <v>127608</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B33" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B34" s="2">
-        <v>5</v>
-      </c>
-      <c r="C34" s="2">
-        <v>126739243</v>
-      </c>
-      <c r="D34" s="2">
-        <v>127054568</v>
-      </c>
-      <c r="E34" s="2">
-        <v>315000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B35" s="2">
-        <v>5</v>
-      </c>
-      <c r="C35" s="2">
-        <v>126763765</v>
-      </c>
-      <c r="D35" s="2">
-        <v>126913191</v>
-      </c>
-      <c r="E35" s="2">
-        <v>275540</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B35" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B36" s="2">
-        <v>5</v>
-      </c>
-      <c r="C36" s="2">
-        <v>126766199</v>
-      </c>
-      <c r="D36" s="2">
-        <v>126922932</v>
-      </c>
-      <c r="E36" s="2">
-        <v>156734</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B37" s="2">
-        <v>5</v>
-      </c>
-      <c r="C37" s="2">
-        <v>126762001</v>
-      </c>
-      <c r="D37" s="2">
-        <v>126997121</v>
-      </c>
-      <c r="E37" s="2">
-        <v>235000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B38" s="2">
-        <v>5</v>
-      </c>
-      <c r="C38" s="2">
-        <v>126805047</v>
-      </c>
-      <c r="D38" s="2">
-        <v>126864688</v>
-      </c>
-      <c r="E38" s="2">
-        <v>59651</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B38" s="2" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B39" s="2">
-        <v>5</v>
-      </c>
-      <c r="C39" s="2">
-        <v>126729432</v>
-      </c>
-      <c r="D39" s="2">
-        <v>126915116</v>
-      </c>
-      <c r="E39" s="2">
-        <v>184808</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B40" s="2">
-        <v>5</v>
-      </c>
-      <c r="C40" s="2">
-        <v>126750808</v>
-      </c>
-      <c r="D40" s="2">
-        <v>126903760</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B40" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B41" s="2">
-        <v>5</v>
-      </c>
-      <c r="C41" s="2">
-        <v>126676886</v>
-      </c>
-      <c r="D41" s="2">
-        <v>126896451</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B41" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B42" s="2">
-        <v>5</v>
-      </c>
-      <c r="C42" s="2">
-        <v>126676469</v>
-      </c>
-      <c r="D42" s="2">
-        <v>126897351</v>
-      </c>
-      <c r="E42" s="2">
-        <v>221000</v>
+      <c r="B42" s="2" t="s">
+        <v>261</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>